<commit_message>
Update control_file_msr_creator.xlsx with new data
</commit_message>
<xml_diff>
--- a/1. MSR Creator/control_file_msr_creator.xlsx
+++ b/1. MSR Creator/control_file_msr_creator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\1. MSR Creator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31900DD-BE70-44A4-99E4-8DE3134C96FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC92F70-3BB9-41D0-B7CE-A99936B51BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3705" yWindow="-13410" windowWidth="17175" windowHeight="12060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paths" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="146">
   <si>
     <t>pv_ghi_threshold</t>
   </si>
@@ -122,9 +122,6 @@
     <t>file_name_protected_areas</t>
   </si>
   <si>
-    <t>WPDA_June2021</t>
-  </si>
-  <si>
     <t>file_name_roads</t>
   </si>
   <si>
@@ -456,6 +453,15 @@
   </si>
   <si>
     <t>C:\Users\mastt\OneDrive - VITO\Documents\21_WP1\RawData\model_supply_regions\workflow\inputs\2022 MSR Toolset Inputs</t>
+  </si>
+  <si>
+    <t>file_name_climate_zones</t>
+  </si>
+  <si>
+    <t>koppen_geiger_0p00833333</t>
+  </si>
+  <si>
+    <t>WDPA_October2023</t>
   </si>
 </sst>
 </file>
@@ -908,57 +914,57 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="8" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B2" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="8" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="8" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="8" customFormat="1" ht="75.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B5" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>79</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -981,35 +987,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" s="12">
         <v>5</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3" s="12">
         <v>20</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1020,95 +1026,95 @@
         <v>2700</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="12">
         <v>0</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="12">
         <v>0</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="12">
         <v>0</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>67</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="12">
+        <v>0</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>69</v>
-      </c>
-      <c r="B9" s="12">
-        <v>1</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="12">
+        <v>0</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="B10" s="12">
-        <v>1</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B11" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B12" s="12">
         <v>1</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1131,21 +1137,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" s="6">
         <v>100</v>
@@ -1154,7 +1160,7 @@
         <v>50</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1167,7 +1173,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -1177,13 +1183,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1203,7 +1209,7 @@
         <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1214,7 +1220,7 @@
         <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1225,132 +1231,141 @@
         <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>31</v>
+        <v>143</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>34</v>
+        <v>145</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>113</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="2"/>
+      <c r="C18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1372,13 +1387,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="C1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1416,29 +1431,29 @@
     </row>
     <row r="5" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B5" s="18">
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B6" s="18">
         <v>20</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B7" s="18">
         <v>10</v>
@@ -1455,7 +1470,7 @@
         <v>33</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1504,7 +1519,7 @@
     </row>
     <row r="13" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B13" s="18">
         <v>10</v>
@@ -1515,24 +1530,24 @@
     </row>
     <row r="14" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B15" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1548,7 +1563,7 @@
     </row>
     <row r="17" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B17" s="18">
         <v>4</v>
@@ -1581,35 +1596,35 @@
     </row>
     <row r="20" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B20" s="18">
         <v>5</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" s="18">
         <v>3</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B22" s="18">
         <v>100</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1620,29 +1635,29 @@
         <v>1960000</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1669,51 +1684,51 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B28" s="18">
         <v>5</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B29" s="18">
         <v>0.01</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B30" s="18">
         <v>2000</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="C31" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B32" s="18">
         <v>8760</v>
@@ -1722,7 +1737,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B33" s="18">
         <v>365</v>
@@ -1731,13 +1746,13 @@
     </row>
     <row r="34" spans="1:3" s="8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B34" s="12">
         <v>5</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>